<commit_message>
Add gaming/heat-spreader RAM option and note mixed Oct 17 load
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AuDyZLJ78Mu3VZWkun6PBK
</commit_message>
<xml_diff>
--- a/BW_Scrap_RAM_Purchases.xlsx
+++ b/BW_Scrap_RAM_Purchases.xlsx
@@ -24,12 +24,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="57">
   <si>
     <t xml:space="preserve">B&amp;W Scrap Yard – RAM Purchase Log</t>
   </si>
   <si>
-    <t xml:space="preserve">Fill in the yellow-header columns (A–K, P). Gray-header columns (L–O) calculate automatically. Row 4 is an example – overwrite or delete it.</t>
+    <t xml:space="preserve">Fill in the yellow-header columns (A–K, P). Gray-header columns (L–O) calculate automatically. Row 4 is an example – overwrite or delete it. Tip: if the yard weighs gaming (heat spreader) RAM separately, log it as its own row with the same Receipt #.</t>
   </si>
   <si>
     <t xml:space="preserve">Date</t>
@@ -78,6 +78,12 @@
   </si>
   <si>
     <t xml:space="preserve">Notes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mixed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mixed load incl. gaming RAM w/ aluminum heat spreaders (lower $/lb rate). Split unknown.</t>
   </si>
   <si>
     <t xml:space="preserve">RAM Purchase Summary</t>
@@ -135,9 +141,6 @@
   </si>
   <si>
     <t xml:space="preserve">DDR5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mixed</t>
   </si>
   <si>
     <t xml:space="preserve">Other</t>
@@ -774,7 +777,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="8" style="1" width="11"/>
@@ -783,7 +786,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="14" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -888,7 +891,9 @@
       </c>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
+      <c r="D5" s="7" t="s">
+        <v>18</v>
+      </c>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
@@ -916,7 +921,9 @@
         <f aca="false">IF(OR(J5="",L5="",L5=0),"",J5/L5)</f>
         <v/>
       </c>
-      <c r="P5" s="7"/>
+      <c r="P5" s="7" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6"/>
@@ -15866,7 +15873,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:D503" type="list">
-      <formula1>"DIMM (Desktop),SODIMM (Laptop),Server (ECC/RDIMM),Mixed"</formula1>
+      <formula1>"DIMM (Desktop),Gaming DIMM (Heat Spreader),SODIMM (Laptop),Server (ECC/RDIMM),Mixed"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K4:K503" type="list">
@@ -15901,12 +15908,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" s="13" t="n">
         <f aca="false">COUNT(Purchases!J4:J503)</f>
@@ -15915,7 +15922,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" s="14" t="n">
         <f aca="false">SUM(Purchases!J4:J503)</f>
@@ -15924,7 +15931,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B5" s="15" t="n">
         <f aca="false">SUM(Purchases!H4:H503)</f>
@@ -15933,7 +15940,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B6" s="16" t="n">
         <f aca="false">SUM(Purchases!I4:I503)</f>
@@ -15951,7 +15958,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B8" s="14" t="n">
         <f aca="false">IF(B5=0,0,B4/B5)</f>
@@ -15960,7 +15967,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B9" s="14" t="n">
         <f aca="false">IF(B6=0,0,B4/B6)</f>
@@ -15969,7 +15976,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B10" s="14" t="n">
         <f aca="false">IF(B7=0,0,B4/B7)</f>
@@ -15978,32 +15985,32 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B15" s="13" t="n">
         <f aca="false">COUNTIF(Purchases!C4:C503,A15)</f>
@@ -16028,7 +16035,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B16" s="13" t="n">
         <f aca="false">COUNTIF(Purchases!C4:C503,A16)</f>
@@ -16053,7 +16060,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B17" s="13" t="n">
         <f aca="false">COUNTIF(Purchases!C4:C503,A17)</f>
@@ -16078,7 +16085,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B18" s="13" t="n">
         <f aca="false">COUNTIF(Purchases!C4:C503,A18)</f>
@@ -16103,7 +16110,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="B19" s="13" t="n">
         <f aca="false">COUNTIF(Purchases!C4:C503,A19)</f>
@@ -16128,7 +16135,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B20" s="13" t="n">
         <f aca="false">COUNTIF(Purchases!C4:C503,A20)</f>
@@ -16153,18 +16160,18 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="19" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B24" s="20" t="n">
         <v>2026</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D24" s="19"/>
       <c r="E24" s="19"/>
@@ -16172,23 +16179,23 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E25" s="19"/>
       <c r="F25" s="19"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B26" s="19" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,1,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,1+1,1))</f>
@@ -16207,7 +16214,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B27" s="19" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,2,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,2+1,1))</f>
@@ -16226,7 +16233,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B28" s="19" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,3,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,3+1,1))</f>
@@ -16245,7 +16252,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B29" s="19" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,4,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,4+1,1))</f>
@@ -16264,7 +16271,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B30" s="19" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,5,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,5+1,1))</f>
@@ -16283,7 +16290,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B31" s="19" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,6,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,6+1,1))</f>
@@ -16302,7 +16309,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B32" s="19" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,7,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,7+1,1))</f>
@@ -16321,7 +16328,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B33" s="19" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,8,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,8+1,1))</f>
@@ -16340,7 +16347,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="19" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B34" s="19" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,9,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,9+1,1))</f>
@@ -16359,7 +16366,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="19" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B35" s="19" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,10,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,10+1,1))</f>
@@ -16378,7 +16385,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B36" s="19" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,11,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,11+1,1))</f>
@@ -16397,7 +16404,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B37" s="19" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,12,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,12+1,1))</f>
@@ -16416,7 +16423,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B38" s="23" t="n">
         <f aca="false">SUM(B26:B37)</f>

</xml_diff>

<commit_message>
Log Oct 30 RAM purchase
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AuDyZLJ78Mu3VZWkun6PBK
</commit_message>
<xml_diff>
--- a/BW_Scrap_RAM_Purchases.xlsx
+++ b/BW_Scrap_RAM_Purchases.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
   <si>
     <t xml:space="preserve">B&amp;W Scrap Yard – RAM Purchase Log</t>
   </si>
@@ -99,6 +99,12 @@
   </si>
   <si>
     <t xml:space="preserve">$50/lb; weight calculated as ($915 - $210) / $50.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17 lbs @ $70/lb. Oct 30 total paid $2,640.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">29 lbs @ $50/lb.</t>
   </si>
   <si>
     <t xml:space="preserve">RAM Purchase Summary</t>
@@ -237,7 +243,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
@@ -246,7 +252,6 @@
     <numFmt numFmtId="169" formatCode="General"/>
     <numFmt numFmtId="170" formatCode="#,##0"/>
     <numFmt numFmtId="171" formatCode="#,##0.00"/>
-    <numFmt numFmtId="172" formatCode="\$#,##0.00"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -412,7 +417,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -489,27 +494,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1112,16 +1097,24 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6"/>
+      <c r="A9" s="6" t="n">
+        <v>46325</v>
+      </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
+      <c r="D9" s="7" t="s">
+        <v>18</v>
+      </c>
       <c r="E9" s="7"/>
       <c r="F9" s="7"/>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="9"/>
+      <c r="I9" s="8" t="n">
+        <v>17</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>1190</v>
+      </c>
       <c r="K9" s="7"/>
       <c r="L9" s="10" t="str">
         <f aca="false">IF(OR(E9="",H9=""),"",E9*H9)</f>
@@ -1131,27 +1124,37 @@
         <f aca="false">IF(OR(J9="",H9="",H9=0),"",J9/H9)</f>
         <v/>
       </c>
-      <c r="N9" s="11" t="str">
+      <c r="N9" s="11" t="n">
         <f aca="false">IF(OR(J9="",I9="",I9=0),"",J9/I9)</f>
-        <v/>
+        <v>70</v>
       </c>
       <c r="O9" s="11" t="str">
         <f aca="false">IF(OR(J9="",L9="",L9=0),"",J9/L9)</f>
         <v/>
       </c>
-      <c r="P9" s="7"/>
+      <c r="P9" s="7" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6"/>
+      <c r="A10" s="6" t="n">
+        <v>46325</v>
+      </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
+      <c r="D10" s="7" t="s">
+        <v>21</v>
+      </c>
       <c r="E10" s="7"/>
       <c r="F10" s="7"/>
       <c r="G10" s="7"/>
       <c r="H10" s="7"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="9"/>
+      <c r="I10" s="8" t="n">
+        <v>29</v>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>1450</v>
+      </c>
       <c r="K10" s="7"/>
       <c r="L10" s="10" t="str">
         <f aca="false">IF(OR(E10="",H10=""),"",E10*H10)</f>
@@ -1161,15 +1164,17 @@
         <f aca="false">IF(OR(J10="",H10="",H10=0),"",J10/H10)</f>
         <v/>
       </c>
-      <c r="N10" s="11" t="str">
+      <c r="N10" s="11" t="n">
         <f aca="false">IF(OR(J10="",I10="",I10=0),"",J10/I10)</f>
-        <v/>
+        <v>50</v>
       </c>
       <c r="O10" s="11" t="str">
         <f aca="false">IF(OR(J10="",L10="",L10=0),"",J10/L10)</f>
         <v/>
       </c>
-      <c r="P10" s="7"/>
+      <c r="P10" s="7" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6"/>
@@ -16000,38 +16005,38 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="11"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="13" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B3" s="14" t="n">
         <f aca="false">COUNT(Purchases!J4:J503)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B4" s="15" t="n">
         <f aca="false">SUM(Purchases!J4:J503)</f>
-        <v>1882.5</v>
+        <v>4522.5</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B5" s="16" t="n">
         <f aca="false">SUM(Purchases!H4:H503)</f>
@@ -16040,11 +16045,11 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B6" s="17" t="n">
         <f aca="false">SUM(Purchases!I4:I503)</f>
-        <v>32.1</v>
+        <v>78.1</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16058,7 +16063,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B8" s="15" t="n">
         <f aca="false">IF(B5=0,0,B4/B5)</f>
@@ -16067,16 +16072,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B9" s="15" t="n">
         <f aca="false">IF(B6=0,0,B4/B6)</f>
-        <v>58.6448598130841</v>
+        <v>57.9065300896287</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B10" s="15" t="n">
         <f aca="false">IF(B7=0,0,B4/B7)</f>
@@ -16085,50 +16090,50 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" s="19" t="s">
-        <v>34</v>
+        <v>35</v>
+      </c>
+      <c r="H13" s="18" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="B14" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="20" t="s">
+      <c r="A14" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="B14" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="C14" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="20" t="s">
+      <c r="D14" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="H14" s="21" t="s">
+      <c r="E14" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="I14" s="21" t="s">
+      <c r="F14" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="J14" s="21" t="s">
+      <c r="H14" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="I14" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="J14" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="K14" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="L14" s="21" t="s">
-        <v>43</v>
+      <c r="K14" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="L14" s="19" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B15" s="14" t="n">
         <f aca="false">COUNTIF(Purchases!C4:C503,A15)</f>
@@ -16150,29 +16155,29 @@
         <f aca="false">IF(C15=0,0,E15/C15)</f>
         <v>0</v>
       </c>
-      <c r="H15" s="22" t="s">
+      <c r="H15" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="I15" s="22" t="n">
+      <c r="I15" s="14" t="n">
         <f aca="false">COUNTIF(Purchases!D4:D503,H15)</f>
-        <v>3</v>
-      </c>
-      <c r="J15" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="J15" s="17" t="n">
         <f aca="false">SUMIF(Purchases!D4:D503,H15,Purchases!I4:I503)</f>
-        <v>13.875</v>
-      </c>
-      <c r="K15" s="24" t="n">
+        <v>30.875</v>
+      </c>
+      <c r="K15" s="15" t="n">
         <f aca="false">SUMIF(Purchases!D4:D503,H15,Purchases!J4:J503)</f>
-        <v>971.25</v>
-      </c>
-      <c r="L15" s="24" t="n">
+        <v>2161.25</v>
+      </c>
+      <c r="L15" s="15" t="n">
         <f aca="false">IF(J15=0,0,K15/J15)</f>
         <v>70</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B16" s="14" t="n">
         <f aca="false">COUNTIF(Purchases!C4:C503,A16)</f>
@@ -16194,29 +16199,29 @@
         <f aca="false">IF(C16=0,0,E16/C16)</f>
         <v>0</v>
       </c>
-      <c r="H16" s="22" t="s">
+      <c r="H16" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="I16" s="22" t="n">
+      <c r="I16" s="14" t="n">
         <f aca="false">COUNTIF(Purchases!D4:D503,H16)</f>
-        <v>2</v>
-      </c>
-      <c r="J16" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="J16" s="17" t="n">
         <f aca="false">SUMIF(Purchases!D4:D503,H16,Purchases!I4:I503)</f>
-        <v>18.225</v>
-      </c>
-      <c r="K16" s="24" t="n">
+        <v>47.225</v>
+      </c>
+      <c r="K16" s="15" t="n">
         <f aca="false">SUMIF(Purchases!D4:D503,H16,Purchases!J4:J503)</f>
-        <v>911.25</v>
-      </c>
-      <c r="L16" s="24" t="n">
+        <v>2361.25</v>
+      </c>
+      <c r="L16" s="15" t="n">
         <f aca="false">IF(J16=0,0,K16/J16)</f>
         <v>50</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B17" s="14" t="n">
         <f aca="false">COUNTIF(Purchases!C4:C503,A17)</f>
@@ -16238,29 +16243,29 @@
         <f aca="false">IF(C17=0,0,E17/C17)</f>
         <v>0</v>
       </c>
-      <c r="H17" s="22" t="s">
-        <v>47</v>
-      </c>
-      <c r="I17" s="22" t="n">
+      <c r="H17" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="I17" s="14" t="n">
         <f aca="false">COUNTIF(Purchases!D4:D503,H17)</f>
         <v>0</v>
       </c>
-      <c r="J17" s="23" t="n">
+      <c r="J17" s="17" t="n">
         <f aca="false">SUMIF(Purchases!D4:D503,H17,Purchases!I4:I503)</f>
         <v>0</v>
       </c>
-      <c r="K17" s="24" t="n">
+      <c r="K17" s="15" t="n">
         <f aca="false">SUMIF(Purchases!D4:D503,H17,Purchases!J4:J503)</f>
         <v>0</v>
       </c>
-      <c r="L17" s="24" t="n">
+      <c r="L17" s="15" t="n">
         <f aca="false">IF(J17=0,0,K17/J17)</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B18" s="14" t="n">
         <f aca="false">COUNTIF(Purchases!C4:C503,A18)</f>
@@ -16282,29 +16287,29 @@
         <f aca="false">IF(C18=0,0,E18/C18)</f>
         <v>0</v>
       </c>
-      <c r="H18" s="22" t="s">
-        <v>49</v>
-      </c>
-      <c r="I18" s="22" t="n">
+      <c r="H18" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="I18" s="14" t="n">
         <f aca="false">COUNTIF(Purchases!D4:D503,H18)</f>
         <v>0</v>
       </c>
-      <c r="J18" s="23" t="n">
+      <c r="J18" s="17" t="n">
         <f aca="false">SUMIF(Purchases!D4:D503,H18,Purchases!I4:I503)</f>
         <v>0</v>
       </c>
-      <c r="K18" s="24" t="n">
+      <c r="K18" s="15" t="n">
         <f aca="false">SUMIF(Purchases!D4:D503,H18,Purchases!J4:J503)</f>
         <v>0</v>
       </c>
-      <c r="L18" s="24" t="n">
+      <c r="L18" s="15" t="n">
         <f aca="false">IF(J18=0,0,K18/J18)</f>
         <v>0</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B19" s="14" t="n">
         <f aca="false">COUNTIF(Purchases!C4:C503,A19)</f>
@@ -16326,29 +16331,29 @@
         <f aca="false">IF(C19=0,0,E19/C19)</f>
         <v>0</v>
       </c>
-      <c r="H19" s="22" t="s">
-        <v>50</v>
-      </c>
-      <c r="I19" s="22" t="n">
+      <c r="H19" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="I19" s="14" t="n">
         <f aca="false">COUNTIF(Purchases!D4:D503,H19)</f>
         <v>0</v>
       </c>
-      <c r="J19" s="23" t="n">
+      <c r="J19" s="17" t="n">
         <f aca="false">SUMIF(Purchases!D4:D503,H19,Purchases!I4:I503)</f>
         <v>0</v>
       </c>
-      <c r="K19" s="24" t="n">
+      <c r="K19" s="15" t="n">
         <f aca="false">SUMIF(Purchases!D4:D503,H19,Purchases!J4:J503)</f>
         <v>0</v>
       </c>
-      <c r="L19" s="24" t="n">
+      <c r="L19" s="15" t="n">
         <f aca="false">IF(J19=0,0,K19/J19)</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B20" s="14" t="n">
         <f aca="false">COUNTIF(Purchases!C4:C503,A20)</f>
@@ -16373,285 +16378,285 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="25" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" s="26" t="n">
+      <c r="A24" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" s="21" t="n">
         <v>2026</v>
       </c>
-      <c r="C24" s="27" t="s">
-        <v>54</v>
-      </c>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="25"/>
+      <c r="C24" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="D24" s="20"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="B25" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="D25" s="20" t="s">
+      <c r="A25" s="19" t="s">
+        <v>57</v>
+      </c>
+      <c r="B25" s="19" t="s">
+        <v>44</v>
+      </c>
+      <c r="C25" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25"/>
+      <c r="D25" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="25" t="s">
-        <v>56</v>
-      </c>
-      <c r="B26" s="25" t="n">
+      <c r="A26" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="B26" s="20" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,1,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,1+1,1))</f>
         <v>0</v>
       </c>
-      <c r="C26" s="25" t="n">
+      <c r="C26" s="20" t="n">
         <f aca="false">SUMIFS(Purchases!H4:H503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,1,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,1+1,1))</f>
         <v>0</v>
       </c>
-      <c r="D26" s="28" t="n">
+      <c r="D26" s="23" t="n">
         <f aca="false">SUMIFS(Purchases!J4:J503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,1,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,1+1,1))</f>
         <v>0</v>
       </c>
-      <c r="E26" s="25"/>
-      <c r="F26" s="25"/>
+      <c r="E26" s="20"/>
+      <c r="F26" s="20"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="B27" s="25" t="n">
+      <c r="A27" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="B27" s="20" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,2,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,2+1,1))</f>
         <v>0</v>
       </c>
-      <c r="C27" s="25" t="n">
+      <c r="C27" s="20" t="n">
         <f aca="false">SUMIFS(Purchases!H4:H503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,2,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,2+1,1))</f>
         <v>0</v>
       </c>
-      <c r="D27" s="28" t="n">
+      <c r="D27" s="23" t="n">
         <f aca="false">SUMIFS(Purchases!J4:J503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,2,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,2+1,1))</f>
         <v>0</v>
       </c>
-      <c r="E27" s="25"/>
-      <c r="F27" s="25"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="25" t="s">
-        <v>58</v>
-      </c>
-      <c r="B28" s="25" t="n">
+      <c r="A28" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="B28" s="20" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,3,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,3+1,1))</f>
         <v>0</v>
       </c>
-      <c r="C28" s="25" t="n">
+      <c r="C28" s="20" t="n">
         <f aca="false">SUMIFS(Purchases!H4:H503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,3,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,3+1,1))</f>
         <v>0</v>
       </c>
-      <c r="D28" s="28" t="n">
+      <c r="D28" s="23" t="n">
         <f aca="false">SUMIFS(Purchases!J4:J503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,3,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,3+1,1))</f>
         <v>0</v>
       </c>
-      <c r="E28" s="25"/>
-      <c r="F28" s="25"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="B29" s="25" t="n">
+      <c r="A29" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" s="20" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,4,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,4+1,1))</f>
         <v>0</v>
       </c>
-      <c r="C29" s="25" t="n">
+      <c r="C29" s="20" t="n">
         <f aca="false">SUMIFS(Purchases!H4:H503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,4,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,4+1,1))</f>
         <v>0</v>
       </c>
-      <c r="D29" s="28" t="n">
+      <c r="D29" s="23" t="n">
         <f aca="false">SUMIFS(Purchases!J4:J503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,4,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,4+1,1))</f>
         <v>0</v>
       </c>
-      <c r="E29" s="25"/>
-      <c r="F29" s="25"/>
+      <c r="E29" s="20"/>
+      <c r="F29" s="20"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="25" t="s">
-        <v>60</v>
-      </c>
-      <c r="B30" s="25" t="n">
+      <c r="A30" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" s="20" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,5,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,5+1,1))</f>
         <v>0</v>
       </c>
-      <c r="C30" s="25" t="n">
+      <c r="C30" s="20" t="n">
         <f aca="false">SUMIFS(Purchases!H4:H503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,5,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,5+1,1))</f>
         <v>0</v>
       </c>
-      <c r="D30" s="28" t="n">
+      <c r="D30" s="23" t="n">
         <f aca="false">SUMIFS(Purchases!J4:J503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,5,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,5+1,1))</f>
         <v>0</v>
       </c>
-      <c r="E30" s="25"/>
-      <c r="F30" s="25"/>
+      <c r="E30" s="20"/>
+      <c r="F30" s="20"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="25" t="s">
-        <v>61</v>
-      </c>
-      <c r="B31" s="25" t="n">
+      <c r="A31" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" s="20" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,6,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,6+1,1))</f>
         <v>0</v>
       </c>
-      <c r="C31" s="25" t="n">
+      <c r="C31" s="20" t="n">
         <f aca="false">SUMIFS(Purchases!H4:H503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,6,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,6+1,1))</f>
         <v>0</v>
       </c>
-      <c r="D31" s="28" t="n">
+      <c r="D31" s="23" t="n">
         <f aca="false">SUMIFS(Purchases!J4:J503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,6,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,6+1,1))</f>
         <v>0</v>
       </c>
-      <c r="E31" s="25"/>
-      <c r="F31" s="25"/>
+      <c r="E31" s="20"/>
+      <c r="F31" s="20"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="B32" s="25" t="n">
+      <c r="A32" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="B32" s="20" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,7,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,7+1,1))</f>
         <v>0</v>
       </c>
-      <c r="C32" s="25" t="n">
+      <c r="C32" s="20" t="n">
         <f aca="false">SUMIFS(Purchases!H4:H503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,7,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,7+1,1))</f>
         <v>0</v>
       </c>
-      <c r="D32" s="28" t="n">
+      <c r="D32" s="23" t="n">
         <f aca="false">SUMIFS(Purchases!J4:J503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,7,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,7+1,1))</f>
         <v>0</v>
       </c>
-      <c r="E32" s="25"/>
-      <c r="F32" s="25"/>
+      <c r="E32" s="20"/>
+      <c r="F32" s="20"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="25" t="s">
-        <v>63</v>
-      </c>
-      <c r="B33" s="25" t="n">
+      <c r="A33" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="B33" s="20" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,8,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,8+1,1))</f>
         <v>0</v>
       </c>
-      <c r="C33" s="25" t="n">
+      <c r="C33" s="20" t="n">
         <f aca="false">SUMIFS(Purchases!H4:H503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,8,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,8+1,1))</f>
         <v>0</v>
       </c>
-      <c r="D33" s="28" t="n">
+      <c r="D33" s="23" t="n">
         <f aca="false">SUMIFS(Purchases!J4:J503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,8,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,8+1,1))</f>
         <v>0</v>
       </c>
-      <c r="E33" s="25"/>
-      <c r="F33" s="25"/>
+      <c r="E33" s="20"/>
+      <c r="F33" s="20"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="25" t="s">
-        <v>64</v>
-      </c>
-      <c r="B34" s="25" t="n">
+      <c r="A34" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="B34" s="20" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,9,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,9+1,1))</f>
         <v>0</v>
       </c>
-      <c r="C34" s="25" t="n">
+      <c r="C34" s="20" t="n">
         <f aca="false">SUMIFS(Purchases!H4:H503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,9,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,9+1,1))</f>
         <v>0</v>
       </c>
-      <c r="D34" s="28" t="n">
+      <c r="D34" s="23" t="n">
         <f aca="false">SUMIFS(Purchases!J4:J503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,9,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,9+1,1))</f>
         <v>0</v>
       </c>
-      <c r="E34" s="25"/>
-      <c r="F34" s="25"/>
+      <c r="E34" s="20"/>
+      <c r="F34" s="20"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="25" t="s">
-        <v>65</v>
-      </c>
-      <c r="B35" s="25" t="n">
+      <c r="A35" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="B35" s="20" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,10,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,10+1,1))</f>
-        <v>5</v>
-      </c>
-      <c r="C35" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="C35" s="20" t="n">
         <f aca="false">SUMIFS(Purchases!H4:H503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,10,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,10+1,1))</f>
         <v>0</v>
       </c>
-      <c r="D35" s="28" t="n">
+      <c r="D35" s="23" t="n">
         <f aca="false">SUMIFS(Purchases!J4:J503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,10,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,10+1,1))</f>
-        <v>1882.5</v>
-      </c>
-      <c r="E35" s="25"/>
-      <c r="F35" s="25"/>
+        <v>4522.5</v>
+      </c>
+      <c r="E35" s="20"/>
+      <c r="F35" s="20"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="25" t="s">
-        <v>66</v>
-      </c>
-      <c r="B36" s="25" t="n">
+      <c r="A36" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="B36" s="20" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,11,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,11+1,1))</f>
         <v>0</v>
       </c>
-      <c r="C36" s="25" t="n">
+      <c r="C36" s="20" t="n">
         <f aca="false">SUMIFS(Purchases!H4:H503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,11,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,11+1,1))</f>
         <v>0</v>
       </c>
-      <c r="D36" s="28" t="n">
+      <c r="D36" s="23" t="n">
         <f aca="false">SUMIFS(Purchases!J4:J503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,11,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,11+1,1))</f>
         <v>0</v>
       </c>
-      <c r="E36" s="25"/>
-      <c r="F36" s="25"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="20"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="25" t="s">
-        <v>67</v>
-      </c>
-      <c r="B37" s="25" t="n">
+      <c r="A37" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B37" s="20" t="n">
         <f aca="false">COUNTIFS(Purchases!A4:A503,"&gt;="&amp;DATE($B$24,12,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,12+1,1))</f>
         <v>0</v>
       </c>
-      <c r="C37" s="25" t="n">
+      <c r="C37" s="20" t="n">
         <f aca="false">SUMIFS(Purchases!H4:H503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,12,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,12+1,1))</f>
         <v>0</v>
       </c>
-      <c r="D37" s="28" t="n">
+      <c r="D37" s="23" t="n">
         <f aca="false">SUMIFS(Purchases!J4:J503,Purchases!A4:A503,"&gt;="&amp;DATE($B$24,12,1),Purchases!A4:A503,"&lt;"&amp;DATE($B$24,12+1,1))</f>
         <v>0</v>
       </c>
-      <c r="E37" s="25"/>
-      <c r="F37" s="25"/>
+      <c r="E37" s="20"/>
+      <c r="F37" s="20"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="29" t="s">
-        <v>68</v>
-      </c>
-      <c r="B38" s="29" t="n">
+      <c r="A38" s="24" t="s">
+        <v>70</v>
+      </c>
+      <c r="B38" s="24" t="n">
         <f aca="false">SUM(B26:B37)</f>
-        <v>5</v>
-      </c>
-      <c r="C38" s="29" t="n">
+        <v>7</v>
+      </c>
+      <c r="C38" s="24" t="n">
         <f aca="false">SUM(C26:C37)</f>
         <v>0</v>
       </c>
-      <c r="D38" s="30" t="n">
+      <c r="D38" s="25" t="n">
         <f aca="false">SUM(D26:D37)</f>
-        <v>1882.5</v>
-      </c>
-      <c r="E38" s="29"/>
-      <c r="F38" s="29"/>
+        <v>4522.5</v>
+      </c>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>